<commit_message>
Align assignment with provided automation files
</commit_message>
<xml_diff>
--- a/Manual Test Cases for Option 2.xlsx
+++ b/Manual Test Cases for Option 2.xlsx
@@ -2,24 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="719" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Manual Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sample Template for Option 2" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Manual Test Cases'!$A$1:$G$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sample Template for Option 2'!$A$1:$G$36</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,21 +27,31 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Times New Roman"/>
+      <family val="1"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FF000000"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Iskoola Pota"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -55,7 +64,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -63,29 +72,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -168,44 +198,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -232,14 +262,15 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -266,6 +297,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -277,166 +309,142 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
@@ -447,21 +455,21 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="54" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30.6" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TC ID</t>
+          <t>Test Case ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -495,1296 +503,1296 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="64.95" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Neg_0002</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Image resizing</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Upload a non-image .txt file in the Resize Image upload area.</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>The system should reject the unsupported file and display a clear validation message.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>The file was not rendered in the preview area, but no clear validation message was displayed.</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>It is assumed that unsupported file uploads should always show a user-readable validation message.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3" ht="64.95" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Neg_0003</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Image resizing</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Upload a PNG image larger than the stated 20 MB maximum size.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>The system should reject the oversized image and explain that the maximum size is 20 MB.</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>The image was not accepted for processing and the user remained on the upload screen.</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>The upload panel states that the maximum supported size is 20 MB.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Pos_0004</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Document conversion</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Use Image -&gt; PDF with a valid PNG image.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>The selected image should be accepted and converted into a downloadable PDF.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>The upload was accepted and PDF conversion controls became available.</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>A valid PNG image is considered a supported source file for Image -&gt; PDF conversion.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Neg_0005</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Document conversion</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Use PDF -&gt; Word and upload a PNG file.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>The system should reject the PNG file because PDF -&gt; Word requires a PDF input.</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>The unsupported file was not converted, and no Word output was generated.</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>The feature name indicates that only PDF input should be processed.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Neg_0006</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Document conversion</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Use Word -&gt; PDF and upload a corrupted DOCX file.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>The system should stop conversion and display an error message.</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>The conversion did not complete and no PDF download was produced.</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>A corrupted DOCX cannot be reliably converted into PDF.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Neg_0007</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Document conversion</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Use Image -&gt; PDF and upload an image larger than 20 MB.</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>The system should reject the file and explain the upload limit.</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>The file was not processed for PDF conversion.</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>The same file size limit shown in the upload component should apply to document conversion uploads.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Pos_0008</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>PDF editing</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Open PDF Editor and upload a valid PDF file.</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>The PDF should load into the editor preview with editing controls available.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>The PDF editor accepted the file and displayed editing controls.</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>A normal, unprotected PDF is valid input for the PDF Editor.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Neg_0009</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>PDF editing</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Upload a .txt file into the PDF Editor.</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>The system should reject the non-PDF file and display a validation message.</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>The editor did not display a PDF preview for the unsupported file.</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>The PDF Editor should process PDF files only.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Neg_0010</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>PDF editing</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Upload a corrupted PDF file into the PDF Editor.</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>The system should show an error and prevent editing of the corrupted file.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>The corrupted file was not displayed as an editable PDF.</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>A corrupted PDF cannot be rendered safely for editing.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Neg_0011</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>PDF editing</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Try to save or download from PDF Editor before loading a PDF.</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Save or download actions should be disabled or blocked until a PDF is loaded.</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>No editable document was available and no output file was created.</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Document editing actions should require an uploaded PDF.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Pos_0012</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Use Crop PNG with a valid PNG image and select a crop area.</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>The image preview should appear, the crop area should be adjustable, and cropped output should be downloadable.</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>The image was accepted and crop controls were available for preview and download.</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>A valid PNG is supported by the Crop PNG workflow.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Neg_0013</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Upload a .txt file to the crop tool.</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>The system should reject the unsupported file type and display a validation message.</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>The unsupported file was not displayed in the crop preview.</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Only image files should be accepted by crop tools.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Neg_0014</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Enter zero or negative crop dimensions.</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>The system should prevent invalid crop dimensions and keep the output unavailable.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>The crop output was not generated for invalid dimensions.</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Crop width and height must be positive values.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Neg_0015</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Open the crop tool without uploading an image.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>The preview should show no image and crop/download actions should not create an output.</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>No crop preview or output was produced before an image was uploaded.</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Cropping requires a source image.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Pos_0016</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Compression</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Use PNG Compressor with a valid PNG image.</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>The image should be accepted and a compressed PNG should become downloadable.</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>The PNG was accepted and compression controls were shown.</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>A valid PNG is supported by the PNG Compressor feature.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Neg_0017</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Compression</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Upload a DOCX file to an image compression tool.</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>The system should reject the non-image file and display a validation message.</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>The DOCX file was not processed as an image.</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Compression tools should only process supported image formats.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Neg_0018</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Compression</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Upload an image larger than 20 MB to the compressor.</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>The system should reject the oversized image and display the size limit.</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>The oversized file was not compressed.</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>The upload component advertises a 20 MB maximum file size.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Neg_0019</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Compression</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Attempt to download compressed output before uploading an image.</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Download should be unavailable until an image has been processed.</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>No compressed output was downloaded before an image was uploaded.</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Compression requires a source image.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Pos_0020</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Image format conversion</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Convert a valid PNG image to JPG.</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>The image should be accepted and a JPG output should be downloadable.</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>The PNG was accepted and JPG conversion controls became available.</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>PNG to JPG is a normal supported image conversion path.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Neg_0021</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Image format conversion</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Upload a PDF file to an image converter.</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>The system should reject the PDF because it is not a supported image input.</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>The PDF was not converted into an image output.</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Image conversion tools should not accept document files as image input.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Neg_0022</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Image format conversion</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Upload a corrupted image file to the converter.</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>The system should show an error and avoid creating a converted output.</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>No converted image was generated from the corrupted file.</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>A corrupted image cannot be decoded for conversion.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Neg_0023</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Image format conversion</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Open an image conversion page and try to download without uploading a file.</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>The system should keep download unavailable until a valid source image is uploaded.</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>No output file was downloaded before a source image was selected.</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>Conversion requires a source image.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Pos_0024</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Meme generation</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Upload a PNG image and enter top and bottom meme text.</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>The preview should display the image with the entered text and allow download.</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>The meme image was accepted and text controls were available for generating the preview.</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>Meme generation requires a valid image and text input.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Neg_0025</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Meme generation</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Upload a .txt file to the Meme Generator.</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>The system should reject the file and display a validation message.</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>The text file was not displayed as a meme preview.</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>The meme generator should accept image files only.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Neg_0026</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Meme generation</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Try to generate or download a meme without uploading an image.</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>The system should block output generation until an image is uploaded.</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>No meme preview or output file was created without a source image.</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>A source image is required before meme generation.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Pos_0027</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Color picker</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Upload a valid PNG image and click a colored area.</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>The selected color value should be displayed to the user.</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>The image was accepted and the selected color value was shown in the tool.</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>A valid image is required so the picker can sample pixel color values.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Neg_0028</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Color picker</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Open Color Picker and click the empty preview area before uploading an image.</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>The system should not return a color value before an image is available.</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>No selected image color value was generated before upload.</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>A color value should only be returned from an uploaded image.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Neg_0029</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Color picker</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Upload a non-image .txt file to Color Picker.</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>The system should reject the file and display a validation message.</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>The unsupported file was not shown as an image for color selection, but the validation feedback was not clear.</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>Unsupported uploads should show a clear validation message.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Pos_0030</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>Color picker</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Select two different points from a valid uploaded PNG image.</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>The displayed color value should update after each selection.</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>The selected color value updated when a new point was selected.</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>Different points in the image can contain different colors.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Pos_0031</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Image rotation</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Upload a PNG image and apply a 90 degree rotation.</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>The preview should show the image rotated and output should be downloadable.</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>The image was accepted and rotation controls were available.</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>A valid PNG image is supported by the rotation feature.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Neg_0032</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Image rotation</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Upload a .txt file to the rotation tool.</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>The system should reject the unsupported file and show validation feedback.</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>The text file was not rendered in the rotation preview.</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>Rotation should be available only for supported image files.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Neg_0033</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Image rotation</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Click rotate before uploading an image.</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>The system should prevent rotation and avoid creating output.</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>No rotated image output was created before upload.</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>Rotation requires a source image.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Pos_0034</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>Image flipping</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Upload a PNG image and apply horizontal flip.</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>The preview should show the flipped image and output should be downloadable.</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>The image was accepted and flip controls were available.</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>A valid PNG image is supported by the flip feature.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Neg_0035</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>Image flipping</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Upload a .txt file to the flip tool.</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>The system should reject the unsupported file and show validation feedback.</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>The text file was not rendered in the flip preview.</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>Flip should be available only for supported image files.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Neg_0036</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>Image flipping</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Click flip before uploading an image.</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>The system should prevent the action and avoid creating output.</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t>No flipped image output was created before upload.</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
         <is>
           <t>Image flipping requires a source image.</t>
         </is>
@@ -1792,6 +1800,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G36"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>